<commit_message>
walk through protein contrasts once for every grouping, outputs unchanged
</commit_message>
<xml_diff>
--- a/03_Group_comparisons/Proteome/01_Design_Contrasts/c_data/design_contrasts_all_inputs.xlsx
+++ b/03_Group_comparisons/Proteome/01_Design_Contrasts/c_data/design_contrasts_all_inputs.xlsx
@@ -234,31 +234,31 @@
     <t>03_Group_comparisons/Proteome/01_Design_Contrasts/T1/c_data/design_contrasts.xlsx</t>
   </si>
   <si>
-    <t>52c1ea729f95e38b647c71323efae263</t>
+    <t>a76584ee8c5314e0e09f4da58f76f8ec</t>
   </si>
   <si>
     <t>03_Group_comparisons/Proteome/01_Design_Contrasts/T2/c_data/design_contrasts.xlsx</t>
   </si>
   <si>
-    <t>2452fe7a45dd4d8a48d453b428e4c3d1</t>
+    <t>c02c699bec257e2782fa3b0865ebb354</t>
   </si>
   <si>
     <t>03_Group_comparisons/Proteome/01_Design_Contrasts/T3/c_data/design_contrasts.xlsx</t>
   </si>
   <si>
-    <t>9036fd476850de1091fe54458a5a5675</t>
+    <t>c6ae52c0642b776b880f42492c5c816c</t>
   </si>
   <si>
     <t>03_Group_comparisons/Proteome/01_Design_Contrasts/training/c_data/design_contrasts.xlsx</t>
   </si>
   <si>
-    <t>1104ec2e701808492db73927a3dc6ed6</t>
+    <t>4dcf61d4ec94ec5cd8708e6658360f27</t>
   </si>
   <si>
     <t>03_Group_comparisons/Proteome/01_Design_Contrasts/acute/c_data/design_contrasts.xlsx</t>
   </si>
   <si>
-    <t>865b85c86830087517f2832bfbd38266</t>
+    <t>44d030894b1869a78135f22adcdd22ce</t>
   </si>
   <si>
     <t>BiocGenerics</t>

</xml_diff>

<commit_message>
rebuild every output from scratch; same numbers, fresher timestamps
</commit_message>
<xml_diff>
--- a/03_Group_comparisons/Proteome/01_Design_Contrasts/c_data/design_contrasts_all_inputs.xlsx
+++ b/03_Group_comparisons/Proteome/01_Design_Contrasts/c_data/design_contrasts_all_inputs.xlsx
@@ -234,31 +234,31 @@
     <t>03_Group_comparisons/Proteome/01_Design_Contrasts/T1/c_data/design_contrasts.xlsx</t>
   </si>
   <si>
-    <t>a76584ee8c5314e0e09f4da58f76f8ec</t>
+    <t>dffb191e7e2bc56662a28fa316115821</t>
   </si>
   <si>
     <t>03_Group_comparisons/Proteome/01_Design_Contrasts/T2/c_data/design_contrasts.xlsx</t>
   </si>
   <si>
-    <t>c02c699bec257e2782fa3b0865ebb354</t>
+    <t>2086eac80332c34a730d7e09bd3c4770</t>
   </si>
   <si>
     <t>03_Group_comparisons/Proteome/01_Design_Contrasts/T3/c_data/design_contrasts.xlsx</t>
   </si>
   <si>
-    <t>c6ae52c0642b776b880f42492c5c816c</t>
+    <t>70c199ff6cde75758e8f36557035b95f</t>
   </si>
   <si>
     <t>03_Group_comparisons/Proteome/01_Design_Contrasts/training/c_data/design_contrasts.xlsx</t>
   </si>
   <si>
-    <t>4dcf61d4ec94ec5cd8708e6658360f27</t>
+    <t>e702ed7d1de9cb6012d8a0ab26fbd3a4</t>
   </si>
   <si>
     <t>03_Group_comparisons/Proteome/01_Design_Contrasts/acute/c_data/design_contrasts.xlsx</t>
   </si>
   <si>
-    <t>44d030894b1869a78135f22adcdd22ce</t>
+    <t>9725c5080f07feb470dfb53efa43314b</t>
   </si>
   <si>
     <t>BiocGenerics</t>

</xml_diff>